<commit_message>
Add Sector Fund Type cleaner; extend codebook
scripts/clean_sector_fund_type.R:
- National rollup, NOT per-LG -- no lgcode join.
- Walks rows with a state machine: first occurrence of each sector name
  is the rollup row (dropped); subsequent occurrences are subsectors (kept).
- Drops grand total row (कुल जम्मा).
- Output: 43 rows (11 econ + 8 social + 7 infra + 15 gov + 2 admin) x 14 cols.
- QC: row count matches expected; no NA in sector/subsector cols.

scripts/build_codebook.R:
- Adds Sector Fund Type block: fund types (current/capital/financing/total),
  measures (bud/exp/exp_pct/balance), and dropped row markers.
</commit_message>
<xml_diff>
--- a/docs/codebook.xlsx
+++ b/docs/codebook.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1582,6 +1582,276 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Sector Fund Type</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>fund_type</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>चालु</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>current/recurrent</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Sector Fund Type</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>fund_type</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>पूँजीगत</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>capital</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>capital spending</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Sector Fund Type</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>fund_type</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>वित्तीय</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>financing</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>financing</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Sector Fund Type</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>fund_type</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>जम्मा</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>row total across fund types</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Sector Fund Type</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>measure</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>बजेट</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>bud</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Sector Fund Type</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>measure</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>खर्च</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>exp</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>expenditure</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Sector Fund Type</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>measure</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>खर्च(%)</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>exp_pct</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>expense %</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Sector Fund Type</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>measure</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>मौज्दात</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>closing balance</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Sector Fund Type</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>id_col</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>शीर्षक</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>(split)</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>split into sector + subsector</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Sector Fund Type</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>id_col</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>कुल जम्मा</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>(dropped)</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>grand total row</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Sector Monthly Exp cleaner; extend codebook
scripts/clean_sector_monthly_exp.R:
- National rollup, NOT per-LG.
- Same row state machine as Fund Type (drop sector rollups + grand total).
- 12 monthly expenditure cols (साउन..असार -> exp_saun..exp_asar),
  annual_bud, exp_total, exp_pct, balance.
- QC verified: 43 rows × 20 cols, sector breakdown matches.
- Validates month headers in row 6 cols 4-15 against expected order.

Codebook: +14 Sector Monthly Exp rows (12 months + annual_bud + exp_total).

Note: source data has minor inconsistencies between sum-of-months and
the exp_total column (median diff ~0, max ~44M out of trillions);
preserved as-is.
</commit_message>
<xml_diff>
--- a/docs/codebook.xlsx
+++ b/docs/codebook.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E64"/>
+  <dimension ref="A1:E78"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1852,6 +1852,384 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Sector Monthly Exp</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>साउन</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>exp_saun</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Nepali FY month 1 (mid Jul-Aug)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Sector Monthly Exp</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>भदौ</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>exp_bhadau</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>month 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Sector Monthly Exp</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>आस्बिन</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>exp_asoj</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>month 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Sector Monthly Exp</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>कार्तिक</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>exp_kartik</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>month 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Sector Monthly Exp</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>मार्ग</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>exp_mangsir</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>month 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Sector Monthly Exp</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>पौष</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>exp_poush</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>month 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Sector Monthly Exp</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>माघ</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>exp_magh</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>month 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Sector Monthly Exp</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>फागुन</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>exp_falgun</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>month 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Sector Monthly Exp</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>चैत्र</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>exp_chaitra</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>month 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Sector Monthly Exp</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>बैशाख</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>exp_baisakh</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>month 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Sector Monthly Exp</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>जेठ</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>exp_jestha</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>month 11</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Sector Monthly Exp</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>असार</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>exp_asar</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>month 12 (Jun-mid Jul)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Sector Monthly Exp</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>measure</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>बजेट</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>annual_bud</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>annual budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Sector Monthly Exp</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>measure</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>जम्मा</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>exp_total</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>sum of months (may not match exactly due to source data)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add LG Line Item cleaner (6 FYs, long format); extend codebook
scripts/clean_lg_line_item.R:
- Walks every FY subfolder under "खर्च शीर्षक अनुसार बजेट तथा खर्च/LG Line Item/"
  and writes one output per FY (lg_line_item_fy207677.xlsx etc.).
- Per-file column counts vary (192-216); script auto-detects चालु /
  पूंजीगत / जम्मा group ranges from row 5 so it adapts.
- LONG format (much tidier than 200+ wide cols): one row per
  (LG, line_item) with fund_type ∈ {current, capital} + bud + exp.
- Parses province + district filter from R4C1 title row (files are
  partitioned by district within each FY).
- QC across all 6 FYs: 0 unmatched lgcodes, ~100 distinct line items
  each, all bud/exp populated.

Codebook: +13 entries for LG Line Item (province, district_filter,
line_item code semantics, fund_type levels, etc.).
</commit_message>
<xml_diff>
--- a/docs/codebook.xlsx
+++ b/docs/codebook.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F312"/>
+  <dimension ref="A1:F325"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -10338,6 +10338,422 @@
         </is>
       </c>
     </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>LG Line Item</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>lg_line_item_fy&lt;YYYY&gt;.xlsx</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>id_col</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>(parsed from R4C1)</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>fy</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>Nepali fiscal year (YYYY/YY) parsed from the title row</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>LG Line Item</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>lg_line_item_fy&lt;YYYY&gt;.xlsx</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>id_col</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>प्रदेश</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>province</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>Province name parsed from the title row (files are partitioned by province + district)</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>LG Line Item</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>lg_line_item_fy&lt;YYYY&gt;.xlsx</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>id_col</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>जिल्ला</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>district_filter</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>District name parsed from the title row (the district that this source file represents)</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>LG Line Item</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>lg_line_item_fy&lt;YYYY&gt;.xlsx</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>id_col</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>संकेत</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>lg_code_raw</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>8-digit LG code from source</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>LG Line Item</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>lg_line_item_fy&lt;YYYY&gt;.xlsx</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>id_col</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>स्थानीय तह नाम</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>lg_name_np</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>Full LG name; split into mun_np + district_np</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>LG Line Item</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>lg_line_item_fy&lt;YYYY&gt;.xlsx</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>id_col</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>क्र.सं.</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>(dropped)</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>Serial number</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>LG Line Item</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>lg_line_item_fy&lt;YYYY&gt;.xlsx</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>id_col</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>जम्मा (row)</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>(dropped)</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>Grand-total row at bottom of source</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>LG Line Item</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>lg_line_item_fy&lt;YYYY&gt;.xlsx</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>id_col</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>जम्मा (col block)</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>(dropped)</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>Grand-total column block at right of source</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>LG Line Item</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>lg_line_item_fy&lt;YYYY&gt;.xlsx</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>fund_type</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>चालु</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>Current (recurrent) expenditure line items -- codes typically start with 2xxxx</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>LG Line Item</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>lg_line_item_fy&lt;YYYY&gt;.xlsx</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>fund_type</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>पूंजीगत</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>capital</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>Capital expenditure line items -- codes typically start with 3xxxx</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>LG Line Item</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>lg_line_item_fy&lt;YYYY&gt;.xlsx</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>measure</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>बजेट</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>bud</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>Budget for the line item</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>LG Line Item</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>lg_line_item_fy&lt;YYYY&gt;.xlsx</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>measure</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>खर्च</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>exp</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>Expenditure for the line item</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>LG Line Item</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>lg_line_item_fy&lt;YYYY&gt;.xlsx</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>id_col</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>(line item code)</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>line_item</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>Government chart-of-accounts code (e.g. 21111 = compensation of employees, 22xxx = goods &amp; services, 31xxx = fixed capital, etc.). The data is LONG-format: one row per (LG, line item). First digit indicates fund type (see fund_type col).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add LG Kosh + LG Summary cleaners; extend codebook
clean_lg_kosh.R:
- Per-LG budget vs expenditure across 12 special funds (कोष) like
  contingency, employee welfare, disaster, women & child, etc.
- Drops grand-total fund column (C28-29) and totals row.
- QC: 699 rows × 31 cols, 0 unmatched lgcodes.

clean_lg_summary.R:
- Per-LG operational fund summary (single-row flat header).
- Parses negative values from (parentheses) form.
- QC: 691 rows × 12 cols, 0 unmatched lgcodes.

Codebook +22 entries documenting all 12 funds + opening/closing balance
+ receipts/expenditure flow.
</commit_message>
<xml_diff>
--- a/docs/codebook.xlsx
+++ b/docs/codebook.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F325"/>
+  <dimension ref="A1:F347"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -10754,6 +10754,710 @@
         </is>
       </c>
     </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>LG Kosh</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>lg_kosh.xlsx</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>fund</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>आकस्मिक कोष</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>contingency</t>
+        </is>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>Contingency Fund — money set aside for unforeseen expenses</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>LG Kosh</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>lg_kosh.xlsx</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>fund</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>कर्मचारी कल्याण कोष</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>emp_welfare</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>Employee Welfare Fund — benefits / welfare for LG staff</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>LG Kosh</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>lg_kosh.xlsx</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>fund</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>कार्य संचालन कोष - बिबिध</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>ops_misc</t>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>Operations Fund (Miscellaneous) — general operations spending</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>LG Kosh</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>lg_kosh.xlsx</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>fund</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>गरिवी निवारण तथा सामाजिक परिचालन कोष</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>poverty_social</t>
+        </is>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>Poverty Alleviation &amp; Social Mobilization Fund</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>LG Kosh</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>lg_kosh.xlsx</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>fund</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>प्रकोप व्यवस्थापन कोष</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>disaster</t>
+        </is>
+      </c>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>Disaster Management Fund — emergency response &amp; relief</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>LG Kosh</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>lg_kosh.xlsx</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>fund</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>बिबिध खर्च खाता/कोष- बैंक (ग २-७)</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>misc_bank</t>
+        </is>
+      </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>Miscellaneous Expense Account / Fund (Bank Group 2-7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>LG Kosh</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>lg_kosh.xlsx</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>fund</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>मर्मत सम्भार कोष</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>maintenance</t>
+        </is>
+      </c>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>Maintenance Fund — for asset upkeep &amp; repairs</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>LG Kosh</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>lg_kosh.xlsx</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>fund</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>महिला तथा वाल विकास कोष</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>women_child</t>
+        </is>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>Women &amp; Child Development Fund</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>LG Kosh</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>lg_kosh.xlsx</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>fund</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>मानव संशाधन विकास कोष</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>hrd_fund</t>
+        </is>
+      </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>Human Resource Development Fund</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>LG Kosh</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>lg_kosh.xlsx</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>fund</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>वातावरण ब्यवस्थापन कोष</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>env_mgmt</t>
+        </is>
+      </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>Environmental Management Fund</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>LG Kosh</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>lg_kosh.xlsx</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>fund</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>स्थानीय विकास कोष कार्यक्रम संचालन कोष</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>ldf_ops</t>
+        </is>
+      </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>Local Development Fund Program Operations Fund</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>LG Kosh</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>lg_kosh.xlsx</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>fund</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>स्थानीय विकास घुम्ती कोष</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>ldf_revolving</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>Local Development Revolving Fund</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>LG Kosh</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>lg_kosh.xlsx</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>fund</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>जम्मा</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>(dropped)</t>
+        </is>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>Grand-total fund column at end of source</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>LG Kosh</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>lg_kosh.xlsx</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>measure</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>बजेट</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>&lt;fund&gt;_bud</t>
+        </is>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>Budget allocation per fund</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>LG Kosh</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>lg_kosh.xlsx</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>measure</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>खर्च</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>&lt;fund&gt;_exp</t>
+        </is>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>Expenditure per fund</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>LG Summary</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>lg_summary.xlsx</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>measure</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>शुरुको मौज्दात</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>opening_balance</t>
+        </is>
+      </c>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>Opening balance at start of fiscal year (Operational Fund)</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>LG Summary</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>lg_summary.xlsx</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>measure</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>प्राप्त</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>received</t>
+        </is>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>Funds received during the year (may be negative for adjustments)</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>LG Summary</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>lg_summary.xlsx</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>measure</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>जम्मा प्राप्ती</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>total_receipts</t>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>Total receipts = opening balance + received</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>LG Summary</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>lg_summary.xlsx</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>measure</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>खर्च</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>expenditure</t>
+        </is>
+      </c>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t>Expenditure during the year</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>LG Summary</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>lg_summary.xlsx</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>measure</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>मौज्दात</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>closing_balance</t>
+        </is>
+      </c>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t>Closing balance at end of fiscal year</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>LG Summary</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>lg_summary.xlsx</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>id_col</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>क्र.सं.</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>(dropped)</t>
+        </is>
+      </c>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>Serial number</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>LG Summary</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>lg_summary.xlsx</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>id_col</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>जम्मा (row)</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>(dropped)</t>
+        </is>
+      </c>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>Grand-total row at bottom of source</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>